<commit_message>
feat(observer-mode): Implement read-only user observation mode with audit logging
- Added ObserverMode service to manage the activation and deactivation of the observation mode.
- Introduced ObserverAuditModel for logging actions taken during observation sessions.
- Created observer-mode.php endpoint to handle starting and stopping observation sessions.
- Added observer-banner.php layout to display active observation status.
- Updated user list view to include a button for starting observation mode for eligible users.
- Enhanced permission policies to support read-only access during observation.
- Added SQL scripts for database changes related to observer mode and permissions.
- Implemented integration tests to ensure the integrity of the observer mode functionality.
</commit_message>
<xml_diff>
--- a/files/gelir_gider_sablon.xlsx
+++ b/files/gelir_gider_sablon.xlsx
@@ -1,75 +1,74 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emelc\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10956"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Gelir-Gider Listesi" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
-  <si>
-    <t>Tarih</t>
-  </si>
-  <si>
-    <t>Tip(Gelir/Gider)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Sıra</t>
+  </si>
+  <si>
+    <t>Kayıt Tarihi</t>
+  </si>
+  <si>
+    <t>Tür</t>
+  </si>
+  <si>
+    <t>Hesap Adı</t>
   </si>
   <si>
     <t>Kategori</t>
   </si>
   <si>
-    <t>Hesap Adı</t>
-  </si>
-  <si>
-    <t>Tutar</t>
+    <t>Plaka</t>
+  </si>
+  <si>
+    <t>Ödeme Şekli</t>
+  </si>
+  <si>
+    <t>Banka Adı</t>
+  </si>
+  <si>
+    <t>İşlem Tarihi</t>
+  </si>
+  <si>
+    <t>Tutar (TL)</t>
+  </si>
+  <si>
+    <t>Bakiye (TL)</t>
   </si>
   <si>
     <t>Açıklama</t>
-  </si>
-  <si>
-    <t>11.03.2026</t>
-  </si>
-  <si>
-    <t>GELİR</t>
-  </si>
-  <si>
-    <t>Saha Hizmetleri</t>
-  </si>
-  <si>
-    <t>Mehmet Ali Gökmen</t>
-  </si>
-  <si>
-    <t>Mart ayı ödemesi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
@@ -84,12 +83,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2A9D8F"/>
+        <fgColor rgb="FF135BEC"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -97,19 +96,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -399,33 +423,36 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="6.998" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:12" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -433,30 +460,26 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>1500</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>